<commit_message>
Play-test 14 (lane D): deleted ids out of the source spreadsheets
pt14_xlsx_prune.py edits the workbooks' XML (layout, styles, formulas, cached values kept); report in Docs/fixes.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/ai/Machine_Brigade_AI_Research.xlsx
+++ b/Docs/ai/Machine_Brigade_AI_Research.xlsx
@@ -7675,39 +7675,17 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>377</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>378</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>312</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>313</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>379</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
@@ -7745,39 +7723,17 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>383</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>384</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>312</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>313</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
@@ -8060,74 +8016,30 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>71</v>
-      </c>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>410</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>411</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>93</v>
-      </c>
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
@@ -8725,39 +8637,17 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>455</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>456</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="H37" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="I37" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="J37" s="6" t="s">
-        <v>457</v>
-      </c>
-      <c r="K37" s="6" t="s">
-        <v>242</v>
-      </c>
+      <c r="A37" s="6"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
@@ -8935,39 +8825,17 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="s">
-        <v>467</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="G43" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="H43" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="I43" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="J43" s="6" t="s">
-        <v>370</v>
-      </c>
-      <c r="K43" s="6" t="s">
-        <v>231</v>
-      </c>
+      <c r="A43" s="6"/>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
@@ -9110,39 +8978,17 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="s">
-        <v>476</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>477</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="H48" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="I48" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="J48" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="K48" s="5" t="s">
-        <v>337</v>
-      </c>
+      <c r="A48" s="5"/>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
@@ -9355,39 +9201,17 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="6" t="s">
-        <v>492</v>
-      </c>
-      <c r="B55" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>299</v>
-      </c>
-      <c r="F55" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="G55" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="H55" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="I55" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="J55" s="6" t="s">
-        <v>494</v>
-      </c>
-      <c r="K55" s="6" t="s">
-        <v>304</v>
-      </c>
+      <c r="A55" s="6"/>
+      <c r="B55" s="6"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6"/>
+      <c r="K55" s="6"/>
     </row>
     <row r="56" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">

</xml_diff>